<commit_message>
Tighten external exposure classification
</commit_message>
<xml_diff>
--- a/data/validation/campanella_caleb_blinded_review_completed.xlsx
+++ b/data/validation/campanella_caleb_blinded_review_completed.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R30772521f210415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="2" r:id="Reb33f972e3964c79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer decisions" sheetId="3" r:id="R0d744afb470d4d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="4" r:id="R60033b762a0f468d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re27f414ad1874067"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="2" r:id="Rbcec67e6e6894b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer decisions" sheetId="3" r:id="Re8c7b5ba24f343e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methods" sheetId="4" r:id="Rd1f778f58e614104"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
     <x:numFmt numFmtId="203" formatCode="mm/dd/yyyy"/>
+    <x:numFmt numFmtId="204" formatCode="0.000"/>
   </x:numFmts>
   <x:fonts count="14">
     <x:font>
@@ -97,7 +98,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -122,6 +123,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -245,7 +266,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="174">
+  <x:cellXfs count="188">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -693,6 +714,44 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -922,7 +981,7 @@
   <x:sheetData>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="160" t="str">
-        <x:v>Campanella external transport: blinded human review</x:v>
+        <x:v>Campanella external transport: blinded human review and final adjudication</x:v>
       </x:c>
       <x:c r="B2" s="160"/>
       <x:c r="C2" s="160"/>
@@ -1006,7 +1065,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="107" t="str">
-        <x:v>Exact class agreement</x:v>
+        <x:v>Initial blinded agreement with pre-audit class</x:v>
       </x:c>
       <x:c r="B8" s="106" t="n">
         <x:v>58</x:v>
@@ -1021,7 +1080,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="107" t="str">
-        <x:v>Agreement proportion</x:v>
+        <x:v>Initial agreement proportion</x:v>
       </x:c>
       <x:c r="B9" s="109" t="n">
         <x:v>0.9666666666666667</x:v>
@@ -1036,9 +1095,9 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="107" t="str">
-        <x:v>Unweighted Cohen's kappa</x:v>
-      </x:c>
-      <x:c r="B10" s="109" t="n">
+        <x:v>Initial unweighted Cohen's kappa</x:v>
+      </x:c>
+      <x:c r="B10" s="178" t="n">
         <x:v>0.9475524475524476</x:v>
       </x:c>
       <x:c r="C10" s="106"/>
@@ -1051,10 +1110,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="107" t="str">
-        <x:v>D1 rows upgraded to D2/D3/D4</x:v>
+        <x:v>Agreement with corrected final class</x:v>
       </x:c>
       <x:c r="B11" s="106" t="n">
-        <x:v>0</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C11" s="106"/>
       <x:c r="D11" s="106"/>
@@ -1065,8 +1124,12 @@
       <x:c r="I11" s="106"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="106"/>
-      <x:c r="B12" s="106"/>
+      <x:c r="A12" s="106" t="str">
+        <x:v>Corrected final Cohen's kappa</x:v>
+      </x:c>
+      <x:c r="B12" s="178" t="n">
+        <x:v>0.6037735849056605</x:v>
+      </x:c>
       <x:c r="C12" s="106"/>
       <x:c r="D12" s="106"/>
       <x:c r="E12" s="106"/>
@@ -1076,29 +1139,29 @@
       <x:c r="I12" s="106"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="165" t="str">
-        <x:v>Development class</x:v>
-      </x:c>
-      <x:c r="B13" s="165" t="str">
+      <x:c r="A13" s="187" t="str">
+        <x:v>Corrected final class</x:v>
+      </x:c>
+      <x:c r="B13" s="187" t="str">
         <x:v>Sampled</x:v>
       </x:c>
-      <x:c r="C13" s="165" t="str">
+      <x:c r="C13" s="187" t="str">
         <x:v>Reviewer same class</x:v>
       </x:c>
-      <x:c r="D13" s="165" t="str">
+      <x:c r="D13" s="187" t="str">
         <x:v>Reviewer disagreements</x:v>
       </x:c>
-      <x:c r="E13" s="166"/>
-      <x:c r="F13" s="165" t="str">
-        <x:v>Development \ Reviewer</x:v>
-      </x:c>
-      <x:c r="G13" s="165" t="str">
+      <x:c r="E13" s="183"/>
+      <x:c r="F13" s="187" t="str">
+        <x:v>Corrected final \ Reviewer</x:v>
+      </x:c>
+      <x:c r="G13" s="187" t="str">
         <x:v>D0</x:v>
       </x:c>
-      <x:c r="H13" s="165" t="str">
+      <x:c r="H13" s="187" t="str">
         <x:v>D1</x:v>
       </x:c>
-      <x:c r="I13" s="165" t="str">
+      <x:c r="I13" s="187" t="str">
         <x:v>D2</x:v>
       </x:c>
     </x:row>
@@ -1134,13 +1197,13 @@
         <x:v>D1</x:v>
       </x:c>
       <x:c r="B15" s="111" t="n">
-        <x:v>28</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C15" s="111" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="D15" s="111" t="n">
-        <x:v>2</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E15" s="106"/>
       <x:c r="F15" s="107" t="str">
@@ -1153,35 +1216,19 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="I15" s="106" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="106" t="str">
-        <x:v>D2</x:v>
-      </x:c>
-      <x:c r="B16" s="111" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C16" s="111" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D16" s="111" t="n">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="A16" s="106"/>
+      <x:c r="B16" s="111"/>
+      <x:c r="C16" s="111"/>
+      <x:c r="D16" s="111"/>
       <x:c r="E16" s="106"/>
-      <x:c r="F16" s="107" t="str">
-        <x:v>D2</x:v>
-      </x:c>
-      <x:c r="G16" s="106" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H16" s="106" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I16" s="106" t="n">
-        <x:v>12</x:v>
-      </x:c>
+      <x:c r="F16" s="107"/>
+      <x:c r="G16" s="106"/>
+      <x:c r="H16" s="106"/>
+      <x:c r="I16" s="106"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="106"/>
@@ -1205,18 +1252,18 @@
       <x:c r="H18" s="106"/>
       <x:c r="I18" s="106"/>
     </x:row>
-    <x:row r="19" ht="60" customHeight="1">
-      <x:c r="A19" s="167" t="str">
-        <x:v>Interpretation: The blinded human reviewer agreed on 58 of 60 classes. Both disagreements involved tRes50/ImageNet and the threshold for D0. The reviewer classified these rows as D0; final adjudication retained D1 because the frozen rule requires an explicit version-specific exclusion. No sampled D1 row was upgraded to D2, D3, or D4.</x:v>
-      </x:c>
-      <x:c r="B19" s="168"/>
-      <x:c r="C19" s="168"/>
-      <x:c r="D19" s="168"/>
-      <x:c r="E19" s="168"/>
-      <x:c r="F19" s="168"/>
-      <x:c r="G19" s="168"/>
-      <x:c r="H19" s="168"/>
-      <x:c r="I19" s="169"/>
+    <x:row r="19" ht="72" customHeight="1">
+      <x:c r="A19" s="184" t="str">
+        <x:v>Interpretation: Initial blinded agreement with the pre-audit transport labels was 58/60. A subsequent source-semantics audit found that the 12 Virchow/MSKCC warnings did not establish a containing-corpus relationship, so those rows were conservatively corrected from D2 to D1. Agreement with the corrected final classes was 46/60. Original reviewer decisions remain unchanged.</x:v>
+      </x:c>
+      <x:c r="B19" s="185"/>
+      <x:c r="C19" s="185"/>
+      <x:c r="D19" s="185"/>
+      <x:c r="E19" s="185"/>
+      <x:c r="F19" s="185"/>
+      <x:c r="G19" s="185"/>
+      <x:c r="H19" s="185"/>
+      <x:c r="I19" s="186"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="115"/>
@@ -1287,7 +1334,6 @@
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A19:I21"/>
     <x:mergeCell ref="A23:I25"/>
     <x:mergeCell ref="A19:I19"/>
   </x:mergeCells>
@@ -1334,7 +1380,7 @@
         <x:v>evaluation_institution</x:v>
       </x:c>
       <x:c r="E1" s="165" t="str">
-        <x:v>development_class</x:v>
+        <x:v>preaudit_transport_class</x:v>
       </x:c>
       <x:c r="F1" s="165" t="str">
         <x:v>reviewer_class_original</x:v>
@@ -1361,10 +1407,10 @@
         <x:v>reviewer_source_urls</x:v>
       </x:c>
       <x:c r="N1" s="165" t="str">
-        <x:v>final_adjudicated_class</x:v>
+        <x:v>corrected_final_class</x:v>
       </x:c>
       <x:c r="O1" s="165" t="str">
-        <x:v>resolution</x:v>
+        <x:v>adjudication_or_resolution</x:v>
       </x:c>
       <x:c r="P1" s="165" t="str">
         <x:v>reviewer_identity</x:v>
@@ -1377,6 +1423,9 @@
       </x:c>
       <x:c r="S1" s="165" t="str">
         <x:v>reviewer_used_ai</x:v>
+      </x:c>
+      <x:c r="T1" s="183" t="str">
+        <x:v>agreement_with_corrected_final_class</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -1437,6 +1486,9 @@
       <x:c r="S2" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T2" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="106" t="str">
@@ -1496,6 +1548,9 @@
       <x:c r="S3" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T3" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="106" t="str">
@@ -1555,6 +1610,9 @@
       <x:c r="S4" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T4" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="106" t="str">
@@ -1614,6 +1672,9 @@
       <x:c r="S5" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T5" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="106" t="str">
@@ -1673,6 +1734,9 @@
       <x:c r="S6" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T6" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="106" t="str">
@@ -1732,6 +1796,9 @@
       <x:c r="S7" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T7" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="106" t="str">
@@ -1791,6 +1858,9 @@
       <x:c r="S8" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T8" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="106" t="str">
@@ -1850,6 +1920,9 @@
       <x:c r="S9" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T9" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="106" t="str">
@@ -1909,6 +1982,9 @@
       <x:c r="S10" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T10" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="106" t="str">
@@ -1968,6 +2044,9 @@
       <x:c r="S11" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T11" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="106" t="str">
@@ -2027,6 +2106,9 @@
       <x:c r="S12" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T12" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="106" t="str">
@@ -2086,6 +2168,9 @@
       <x:c r="S13" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T13" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="106" t="str">
@@ -2145,6 +2230,9 @@
       <x:c r="S14" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T14" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="106" t="str">
@@ -2204,6 +2292,9 @@
       <x:c r="S15" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T15" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="106" t="str">
@@ -2263,6 +2354,9 @@
       <x:c r="S16" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T16" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="106" t="str">
@@ -2322,6 +2416,9 @@
       <x:c r="S17" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T17" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="106" t="str">
@@ -2381,6 +2478,9 @@
       <x:c r="S18" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T18" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="106" t="str">
@@ -2440,6 +2540,9 @@
       <x:c r="S19" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T19" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="106" t="str">
@@ -2499,6 +2602,9 @@
       <x:c r="S20" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T20" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="106" t="str">
@@ -2558,6 +2664,9 @@
       <x:c r="S21" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T21" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="106" t="str">
@@ -2617,6 +2726,9 @@
       <x:c r="S22" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T22" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="106" t="str">
@@ -2676,6 +2788,9 @@
       <x:c r="S23" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T23" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="106" t="str">
@@ -2735,6 +2850,9 @@
       <x:c r="S24" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T24" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="106" t="str">
@@ -2794,6 +2912,9 @@
       <x:c r="S25" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T25" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="106" t="str">
@@ -2853,6 +2974,9 @@
       <x:c r="S26" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T26" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="106" t="str">
@@ -2912,6 +3036,9 @@
       <x:c r="S27" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T27" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="106" t="str">
@@ -2971,6 +3098,9 @@
       <x:c r="S28" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T28" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="106" t="str">
@@ -3030,6 +3160,9 @@
       <x:c r="S29" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T29" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="106" t="str">
@@ -3089,6 +3222,9 @@
       <x:c r="S30" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T30" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="106" t="str">
@@ -3148,6 +3284,9 @@
       <x:c r="S31" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T31" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="106" t="str">
@@ -3207,6 +3346,9 @@
       <x:c r="S32" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T32" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="106" t="str">
@@ -3266,6 +3408,9 @@
       <x:c r="S33" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T33" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="106" t="str">
@@ -3325,6 +3470,9 @@
       <x:c r="S34" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T34" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="106" t="str">
@@ -3384,6 +3532,9 @@
       <x:c r="S35" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T35" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="106" t="str">
@@ -3443,6 +3594,9 @@
       <x:c r="S36" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T36" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="106" t="str">
@@ -3502,6 +3656,9 @@
       <x:c r="S37" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T37" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="106" t="str">
@@ -3561,6 +3718,9 @@
       <x:c r="S38" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T38" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="106" t="str">
@@ -3620,6 +3780,9 @@
       <x:c r="S39" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T39" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="106" t="str">
@@ -3679,6 +3842,9 @@
       <x:c r="S40" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T40" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="106" t="str">
@@ -3738,6 +3904,9 @@
       <x:c r="S41" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T41" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="106" t="str">
@@ -3797,6 +3966,9 @@
       <x:c r="S42" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T42" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="106" t="str">
@@ -3839,10 +4011,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N43" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O43" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P43" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -3854,6 +4026,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S43" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T43" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -3898,10 +4073,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N44" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O44" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P44" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -3913,6 +4088,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S44" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T44" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -3957,10 +4135,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N45" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O45" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P45" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -3972,6 +4150,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S45" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T45" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4016,10 +4197,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N46" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O46" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P46" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4031,6 +4212,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S46" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T46" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4075,10 +4259,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N47" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O47" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P47" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4090,6 +4274,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S47" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T47" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4134,10 +4321,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N48" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O48" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P48" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4149,6 +4336,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S48" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T48" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4210,6 +4400,9 @@
       <x:c r="S49" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T49" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="106" t="str">
@@ -4269,6 +4462,9 @@
       <x:c r="S50" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T50" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="106" t="str">
@@ -4328,6 +4524,9 @@
       <x:c r="S51" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T51" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="106" t="str">
@@ -4370,10 +4569,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N52" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O52" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P52" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4385,6 +4584,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S52" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T52" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4429,10 +4631,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N53" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O53" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P53" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4444,6 +4646,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S53" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T53" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4488,10 +4693,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N54" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O54" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P54" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4503,6 +4708,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S54" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T54" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4547,10 +4755,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N55" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O55" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P55" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4562,6 +4770,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S55" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T55" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4606,10 +4817,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N56" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O56" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P56" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4621,6 +4832,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S56" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T56" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4665,10 +4879,10 @@
         <x:v>https://pmc.ncbi.nlm.nih.gov/articles/PMC12003829/; https://github.com/sinai-computational-pathology/SSL_tile_benchmarks/tree/fbdf07f932d7302fd7bcb4a1e6b78bfb9d4a71f9</x:v>
       </x:c>
       <x:c r="N57" s="133" t="str">
-        <x:v>D2_parent_repository_exposure</x:v>
+        <x:v>D1_no_detected_evidence_or_insufficient_disclosure</x:v>
       </x:c>
       <x:c r="O57" s="133" t="str">
-        <x:v>No adjudication required.</x:v>
+        <x:v>Post-review source-semantics audit: same-institution pretraining plus an explicit warning that overlap cannot be excluded does not establish a containing-corpus relationship. Corrected final class is D1; the overlap warning is retained separately.</x:v>
       </x:c>
       <x:c r="P57" s="106" t="str">
         <x:v>Caleb Yitna Ref</x:v>
@@ -4680,6 +4894,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S57" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T57" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4741,6 +4958,9 @@
       <x:c r="S58" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T58" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="106" t="str">
@@ -4800,6 +5020,9 @@
       <x:c r="S59" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T59" s="121" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="106" t="str">
@@ -4859,6 +5082,9 @@
       <x:c r="S60" s="106" t="str">
         <x:v>No</x:v>
       </x:c>
+      <x:c r="T60" s="121" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="106" t="str">
@@ -4916,6 +5142,9 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S61" s="106" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T61" s="121" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -6918,24 +7147,24 @@
       <x:c r="E18" s="119"/>
       <x:c r="F18" s="120"/>
     </x:row>
-    <x:row r="19" ht="54" customHeight="1">
+    <x:row r="19" ht="70" customHeight="1">
       <x:c r="A19" s="105" t="str">
-        <x:v>Adjudication</x:v>
+        <x:v>Post-review source audit</x:v>
       </x:c>
       <x:c r="B19" s="133" t="str">
-        <x:v>Two tRes50 disagreements were reviewed after unblinding. Final D1 was retained because D0 requires an explicit version-specific exclusion; cross-domain/ImageNet provenance alone did not meet that requirement.</x:v>
+        <x:v>After the blind comparison, a source-semantics audit determined that same-institution pretraining plus an explicit warning that overlap cannot be excluded did not establish a containing-corpus relationship. Twelve Virchow/MSKCC rows were corrected from D2 to D1. The explicit overlap warnings and original reviewer decisions were retained.</x:v>
       </x:c>
       <x:c r="C19" s="106"/>
       <x:c r="D19" s="106"/>
       <x:c r="E19" s="106"/>
       <x:c r="F19" s="106"/>
     </x:row>
-    <x:row r="20" ht="54" customHeight="1">
+    <x:row r="20" ht="70" customHeight="1">
       <x:c r="A20" s="157" t="str">
         <x:v>No third adjudicator</x:v>
       </x:c>
       <x:c r="B20" s="158" t="str">
-        <x:v>No third reviewer was used; the two disagreements were resolved by applying the frozen rule.</x:v>
+        <x:v>No third reviewer was used. The two tRes50 disagreements and the 12 D2 boundary corrections were resolved by applying the frozen class definitions to the cited evidence.</x:v>
       </x:c>
       <x:c r="C20" s="158"/>
       <x:c r="D20" s="158"/>

</xml_diff>